<commit_message>
fix(rq3): strip <think> tags from qualitative FP/FN rater sheet (B5)
The XLSX export rendered raw <think> blocks for thinking-mode responses;
apply the same prepare_rater_text stripping used for the LLM judge and the
original rater sheet so reviewers see only the communicated output.
</commit_message>
<xml_diff>
--- a/results/rq3_baseline/rq3_b5_qualitative_cases_rater_sheet.xlsx
+++ b/results/rq3_baseline/rq3_b5_qualitative_cases_rater_sheet.xlsx
@@ -1895,53 +1895,7 @@
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>&lt;think&gt;
-Okay, let's take a look at this code. It's a C++ function called optimize_unflattened_subqueries in the st_select_lex class. The function seems to handle optimizing subqueries in a SQL query, possibly part of a database system like MySQL.
-First, I need to check for any potential vulnerabilities. Common issues in C++ code could include memory leaks, buffer overflows, use of uninitialized variables, or issues with concurrency. But since this is static analysis, I should focus on code patterns that might lead to vulnerabilities.
-Looking at the code structure: there's a loop over SELECT_LEX_UNIT objects, and within that, another loop over SELECT_LEX objects. The function calls various methods on these objects, like optimize(), which might be where the optimization happens.
-One thing that stands out is the use of pointers and possible memory management. For example, the code checks if subquery_predicate is not null before accessing its members. That's good practice. But are there any places where a pointer might be dereferenced without checking?
-Looking at the line: Item_subselect *subquery_predicate= un-&gt;item; Then, if (subquery_predicate) { ... }, so that's safe. Similarly, when casting to Item_in_subselect, they check if it's the right type. So that's okay.
-Another area to check is resource handling. For example, when they call un-&gt;save_union_explain, if that returns true, the function returns true. But what about error handling? If any of these functions return an error, does the code handle it properly?
-Wait, the code has several places where it calls functions like optimize(), and if they return a non-zero value (assuming res is an int and 0 means success), then it returns TRUE. But in C++, TRUE is typically 1, so if res is non-zero, it returns 1. That seems correct for error handling.
-Another thing to check is the use of loops and possible infinite loops. The outer loop is over un, which starts at first_inner_unit() and proceeds via next_unit() or next_unit being set. The inner loop is over sl in un-&gt;first_select(), which seems to process each SELECT_LEX in the unit. The loops don't seem to have obvious infinite loop conditions.
-What about concurrency issues? The code accesses and modifies various member variables of objects like un, sl, inner_join, etc. If this function is called in a multi-threaded context without proper synchronization, there could be race conditions. However, static analysis can't determine if the code is thread-safe unless there are obvious missing locks or shared data structures. Since the code doesn't show any locking mechanisms, but it's part of a database system which might handle that elsewhere, this might not be a vulnerability here.
-Looking for buffer overflows: the code doesn't seem to use any arrays or string operations that could lead to buffer overflows. It's mostly dealing with object pointers and method calls.
-Another possible issue is the handling of the 'next_unit' variable. In the outer loop, the loop condition is 'un; un = next_unit ? next_unit : un-&gt;next_unit();'. So if next_unit is set, it uses that, else it uses the current un's next. But in the code, after processing a subquery, there's a part where if the subquery is fixed, it sets next_unit to un-&gt;next_unit(), then if next_unit exists, it continues, else breaks. That seems okay, but maybe there's a case where next_unit is not properly updated, leading to skipping some units or infinite loops. But without knowing the exact implementation of next_unit() and exclude_level(), it's hard to tell. However, this might be a logic error rather than a vulnerability.
-Another point: when they call un-&gt;set_limit(un-&gt;global_parameters()), this might set a limit on the number of rows processed. If the global_parameters() could be manipulated by an attacker, maybe leading to excessive resource usage. But again, without knowing the context of how these parameters are set, it's hard to say. However, in a database context, this is probably controlled by the query and not directly user-controllable in a way that would cause a DoS.
-Looking at the line: if (options &amp; SELECT_DESCRIBE) { ... }, but where is 'options' defined? Wait, in the code, the function parameters are (bool const_only), but inside the loop, there's a check on 'options &amp; SELECT_DESCRIBE'. Wait, that's a problem. Because 'options' is not declared in the function. Wait, looking at the code again:
-In the code snippet provided, inside the loop over sl, there's:
-if (options &amp; SELECT_DESCRIBE)
-But where is 'options' declared? The function parameters are (bool const_only), and the code doesn't show a variable named 'options' being declared. This could be a typo or a missing variable. Wait, perhaps 'options' is a member variable of the class st_select_lex? Because the function is a member function of st_select_lex, so 'this-&gt;options' might be intended. But if the code as written uses 'options' without qualification, and if that's not a member variable, then this would be a compilation error. However, assuming that the code is correct and compiles, then 'options' must be a member variable. But in the context of static analysis, if 'options' is not properly initialized or controlled, this could lead to incorrect behavior. However, this might not be a vulnerability per se.
-Wait, but the code as presented here might have a bug here. If 'options' is not a member variable, then this code would not compile. But since the user provided this code, perhaps it's correct in context. However, this could be a potential issue if 'options' is not properly set. For example, if the code is checking some option that's not properly validated, leading to incorrect optimization. But again, not sure if this is a vulnerability.
-Another thing to check: the code calls inner_join-&gt;optimize(), which might recursively call optimization functions. If there's a deep recursion here, it could lead to a stack overflow. But again, without knowing the structure of the queries being processed, it's hard to say. However, in a database system, this is probably handled with proper limits.
-Looking for use-after-free or dangling pointers. For example, after calling un-&gt;exclude_level(), which might remove the current unit from some structure, but the code continues to process 'un' in the loop. However, the loop's iteration is controlled by 'un' and 'next_unit', which might be handled correctly. But if exclude_level() modifies the linked list that the loop is traversing, that could lead to issues. For example, if exclude_level() removes 'un' from the list, then the next iteration might have problems. However, in the code, after calling exclude_level(), it sets next_unit to un-&gt;next_unit(), then if next_unit exists, it continues (so skips the rest of the loop body), else breaks. So the loop would proceed to the next unit. But if exclude_level() has already removed 'un' from the list, then un-&gt;next_unit() might not be valid. However, this depends on the implementation of exclude_level() and next_unit(). Since we can't see those functions, it's hard to tell. But this could be a potential issue if the code is modifying the list while iterating over it, leading to use-after-free or invalid pointer access.
-Another possible issue is the handling of the 'un' pointer. In the loop, 'un' is initially set to first_inner_unit(), and then in each iteration, it's updated based on next_unit or un-&gt;next_unit(). If during the processing of a unit (like in the exclude_level() call), the unit is deleted or the list is modified, then the next iteration could be accessing invalid memory. However, the code seems to handle this by setting next_unit before calling exclude_level(), which might be a way to save the next pointer before the current node is removed. For example:
-next_unit = un-&gt;next_unit();
-un-&gt;exclude_level();
-if (next_unit)
-  continue;
-break;
-So here, they save the next_unit before excluding the current unit. Then, if there is a next_unit, they continue (so the loop will pick up next_unit in the next iteration). Otherwise, break. This seems like a safe way to handle removal of the current element during iteration. So this part might be okay.
-Another thing to check: the code calls sl-&gt;update_used_tables() and sl-&gt;update_correlated_cache(), which might modify some internal state. If these functions have side effects that could lead to vulnerabilities, but again, without seeing their implementation, it's hard to tell.
-Looking for any SQL injection possibilities. But this code is part of the query optimization, which is after the query has been parsed and the abstract syntax tree (or similar structure) has been built. So SQL injection would have been handled at the parsing stage, not here. So probably not an issue here.
-What about integer overflows? The code uses ulonglong for save_options, but not sure where that's used. The variables like empty_union_result, is_correlated_unit, etc., are booleans, so no issues there.
-Another possible issue: the code calls inner_join-&gt;optimize(), which might allocate memory or modify data structures. If this function fails (returns non-zero), the code returns TRUE (which I assume indicates an error). But does it clean up any allocated resources? For example, if optimize() allocates memory and then returns an error, does the code leak memory? However, static analysis can't always detect memory leaks unless there's an obvious missing delete. But in the context of a database system, there might be RAII or other cleanup mechanisms in place.
-Looking at the line: if (res) return TRUE; So if optimize() returns an error, the function returns early. But if during the processing of previous SELECT_LEX units, some resources were allocated, they might not be freed. However, again, without knowing the context, it's hard to say. But this could be a resource leak, which is a type of vulnerability (denial of service via memory exhaustion if repeated).
-But the question is whether the code is vulnerable. A resource leak might be considered a vulnerability, but it's not as direct as something like a buffer overflow or code execution.
-Another thing: the code sets un-&gt;set_limit(un-&gt;global_parameters()); which might set a limit on the number of rows processed. If an attacker can control this limit to be very high, it could lead to excessive resource usage. But again, in a database, the user's privileges and query limits would probably restrict this.
-Wait, but looking at the code again, the line is:
-un-&gt;set_limit(un-&gt;global_parameters());
-Assuming that global_parameters() returns some limit value. If this value is not properly validated, it could be set to a very high number, leading to the subquery processing a large number of rows and causing a denial of service. However, this would depend on how global_parameters() is implemented and whether it's user-controllable. If the user can influence this value through their query, then this could be a problem. But in a typical database system, the user can specify LIMIT in their query, which would be handled here. However, the system should have limits on how high that can be set. If the code allows arbitrarily large limits, then it's a potential DoS vector. But again, without knowing the implementation of global_parameters(), it's hard to say. However, this might be a possible vulnerability.
-But wait, the code is part of the optimizer, so perhaps the 'global_parameters()' here refers to parameters of the query, which could be influenced by the user. If the user can set a very high limit, then the subquery could process a lot of data, leading to high CPU or memory usage. However, this is more of a performance issue rather than a vulnerability unless there's no upper bound. But in practice, databases usually have configurable limits to prevent this.
-Another possible issue: the code calls un-&gt;save_union_explain(...), and if that returns true, it returns true (error). But what does save_union_explain do? If it's writing to a file or some output, there could be a path traversal or other file-related vulnerability. But again, without seeing that function, it's hard to tell.
-In summary, after going through the code, I don't see any obvious vulnerabilities like buffer overflows, use-after-free (assuming the list iteration is handled correctly), or SQL injection. The main possible issues could be:
-1. The use of 'options' without declaration in the snippet (but assuming it's a member variable).
-2. Possible resource leaks if optimize() fails and resources aren't cleaned up.
-3. Potential DoS via high resource usage if limits are not enforced.
-But given that this is a code review for vulnerabilities, and without more context, the most likely answer is that there's no obvious vulnerability here. The code seems to handle error checking (like checking if subquery_predicate is null before dereferencing), and the loop handling seems to manage the iteration correctly by saving next_unit before modifying the list.
-Therefore, the answer is probably NO: No vulnerability detected.
-&lt;/think&gt;
-(2) NO: No vulnerability.
+          <t>(2) NO: No vulnerability.
 **Step-by-Step Analysis:**
 1. **Pointer Handling and Null Checks:**
    - The code checks `if (subquery_predicate)` before accessing its members, preventing null pointer dereferences.
@@ -2485,86 +2439,7 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>&lt;think&gt;
-Okay, let's take a look at this code. Hmm, the function is called BinaryBroadcastFiveFold, which suggests it's handling some kind of broadcasting operation in a binary operation, maybe like adding two tensors with different shapes. The code seems to be part of a machine learning framework, possibly TensorFlow Lite given the namespace tflite.
-First, I need to check for any potential security vulnerabilities. Common issues in such code could be buffer overflows, use of uninitialized variables, or incorrect handling of input data leading to out-of-bounds accesses.
-Looking at the parameters: there are several RuntimeShape objects and data pointers. The function starts by switching some parameters between input1 and input2 based on a condition. Then it determines which input data to use based on the broadcast category.
-The main part is the fivefold nested loops. The code has two cases: one when y4 &gt; 1 and another when y4 == 1. Let's check the loop indices and pointer arithmetic.
-In the general case (y4 &gt; 1), there are loops for i0, i1, i2, i3, and then the innermost loop handled by elementwise_f. The pointers input1_data_ptr and input2_data_ptr are incremented based on the loop variables. The elementwise_f is called with y4 elements, and then input2_data_ptr is incremented by y4 each time. Similarly, output_data_ptr is incremented by y4.
-In the special case (y4 == 1), they use scalar_broadcast_f, which takes y3 elements. Here, input2_data_ptr is incremented by y3, and output_data_ptr by y3. Also, input1_data_ptr is incremented by 1 each time.
-Potential issues could be if the loop variables (y0, y1, y2, y3, y4) are not properly validated. For example, if any of these dimensions are zero or negative, but the code uses them in loops. However, in C++, loop conditions with negative values could cause issues, but typically in such code, the shapes are validated before entering the function.
-Another thing to check is whether the pointers are properly bounded. For example, input1_data_ptr and input2_data_ptr are advanced based on the loop variables. If the input shapes are not correctly calculated, this could lead to out-of-bounds accesses.
-Wait, the code uses params.broadcast_shape[0] to [4], which are y0 to y4. These are presumably the broadcasted dimensions. But how are these values determined? The code doesn't show where they come from. If these values are derived from the input shapes without proper validation, there could be issues. However, since this is a function that's part of a larger framework, it's possible that the shapes are validated before this function is called.
-Looking at the loop structures: in the general case, the innermost loop (i3) runs y3 times, and each time, elementwise_f is called with y4 elements. Then input2_data_ptr is advanced by y4. The output_data_ptr is also advanced by y4. Then, after the i3 loop, input1_data_ptr is advanced by y4. Then, after the i2 loop, input2_data_reset is updated to input2_data_ptr, which is then used in the next i1 iteration.
-Wait, in the general case, the input2_data_ptr is set to input2_data_reset at the start of the i1 loop. Then, for each i2, i3, they process y4 elements. The input2_data_ptr is incremented by y4 each time. But input2_data_reset is the starting point for each i1 iteration. So for each i1, the input2_data starts over. That seems correct for broadcasting.
-But what if the input2_data doesn't have enough elements? For example, if the calculated broadcast shape leads to accessing beyond the input2_data's allocated size. But again, this would depend on the prior validation of the shapes.
-Another thing to note is that the code uses the broadcast_shape from the params. The params are either the original or switched based on the broadcast category. The switching swaps input1 and input2 parameters. But the code seems to handle that correctly.
-In the special case where y4 == 1, the scalar_broadcast_f is used. Here, input1_data_ptr is incremented by 1 each time. But in this case, the inner loop is over y3, and each call to scalar_broadcast_f processes y3 elements. So input2_data_ptr is advanced by y3 each time. The input1_data_ptr is advanced by 1 per i3 iteration. Wait, in the loop structure for the special case:
-for (int i2 = 0; i2 &lt; y2; ++i2) {
-  scalar_broadcast_f(y3, params, *input1_data_ptr, input2_data_ptr, output_data_ptr);
-  input2_data_ptr += y3;
-  output_data_ptr += y3;
-  input1_data_ptr += 1;
-}
-So for each i2 iteration, they process y3 elements. The input1_data_ptr is incremented by 1 each time. But since y4 is 1, the input1_data_ptr's stride here is 1 per i3 (but in this case, the loop over i3 is handled inside scalar_broadcast_f). Wait, no, in the special case, the loop over i3 is not present. Instead, scalar_broadcast_f is called with y3, which would handle that dimension. So the code here is combining the i3 loop into the scalar_broadcast_f function.
-But how does this affect the pointers? For each i2, the scalar_broadcast_f is called once, processing y3 elements. Then input2_data_ptr is advanced by y3, and input1_data_ptr by 1. So if input1_data_ptr is supposed to be broadcasted across y3 elements, then each of those elements would use the same input1_data_ptr value. But in this code, they are incrementing input1_data_ptr by 1 each time. Wait, that might be a problem.
-Wait, in the general case, when y4 &gt; 1, the innermost loop (i3) calls elementwise_f with y4 elements. Then input2_data_ptr is advanced by y4, and output_data_ptr by y4. Then, after the i3 loop, input1_data_ptr is advanced by y4. So for each i3 iteration, the input1_data_ptr is not advanced until after the loop. That suggests that for each i3, the same input1_data_ptr is used for all y4 elements. Then, after processing all i3 (y3 times), input1_data_ptr is advanced by y4 * y3? Wait, no. Let me re-examine:
-In the general case:
-for (int i3 = 0; i3 &lt; y3; ++i3) {
-  elementwise_f(y4, ...);
-  input2_data_ptr += y4;
-  output_data_ptr += y4;
-}
-// After the i3 loop:
-input1_data_ptr += y4;
-So for each i3 iteration, the same input1_data_ptr is used. Then, after processing all i3 (y3 times), input1_data_ptr is advanced by y4. So the total advancement for input1_data_ptr per i2 iteration is y4 * y3? No, wait, no. Because the loop over i3 runs y3 times, but input1_data_ptr is only advanced once after the loop. So for each i2 iteration, input1_data_ptr is advanced by y4. Because the loop over i3 doesn't change input1_data_ptr during the loop. So for each i2, the code processes y3 * y4 elements of input1_data_ptr, but the pointer is only advanced by y4. That seems incorrect. Wait, that can't be right. Because if you have y3 iterations, each time processing y4 elements, then the total elements processed for input1 would be y3 * y4. But the pointer is only advanced by y4. That would mean that the same y4 elements are used for each i3 iteration. Which would be correct if input1 is broadcasted along the y3 dimension. Because in broadcasting, the same data is repeated for each element in the broadcasted dimension.
-Ah, right. So in the general case, input1 is broadcasted along the y3 dimension. So for each i3, the same input1_data_ptr is used. Then, after processing all i3 (y3 times), the input1_data_ptr is advanced by y4. So the next i2 iteration would use the next set of y4 elements for input1.
-Similarly, in the special case where y4 == 1, the code uses scalar_broadcast_f. Here, for each i2 iteration, they call scalar_broadcast_f with y3 elements. The input1_data_ptr is a pointer to a single element (since y4 is 1), and it's incremented by 1 after each scalar_broadcast_f call. Wait, but scalar_broadcast_f is supposed to handle broadcasting a scalar (single element) across y3 elements. So in this case, the input1_data_ptr should not be advanced during the scalar broadcast. But in the code, after the scalar_broadcast_f call, input1_data_ptr is incremented by 1. That seems wrong. Because if you're broadcasting a scalar, you should reuse the same element for all y3 elements. But here, the code is advancing the pointer by 1 each time, which would move to the next element, implying that each scalar_broadcast_f call uses a different scalar. But that would not be a broadcast; that would be a strided access.
-Wait, this might be a bug. Let me think again. In the special case, y4 is 1. The code is handling the case where the innermost dimension (y4) is 1, so they combine the y3 loop into the scalar_broadcast_f. The comment says that this handles the case where y4 == 1, and the innermost loop is a single element. But in the code:
-for (int i2 = 0; i2 &lt; y2; ++i2) {
-  scalar_broadcast_f(y3, params, *input1_data_ptr, input2_data_ptr, output_data_ptr);
-  input2_data_ptr += y3;
-  output_data_ptr += y3;
-  input1_data_ptr += 1;
-}
-Here, after each call to scalar_broadcast_f, which processes y3 elements, the input1_data_ptr is incremented by 1. But if this is supposed to be a broadcast, then the same input1 element should be used for all y3 elements. However, the code is advancing the pointer by 1, which would mean that each scalar_broadcast_f call uses a different input1 element. That would not be a broadcast but rather a strided access. This could lead to incorrect results or even out-of-bounds access if the input1_data doesn't have enough elements.
-Wait, but how is this possible? Let's think about the dimensions. The input1.shape.FlatSize is y0 * y1 * y2 * y4 (since y3 is broadcast for input1). But in the special case, y4 is 1, so input1's flat size is y0 * y1 * y2 * 1. The loop variables are i0 (y0), i1 (y1), i2 (y2). So for each i0, i1, i2, the code processes one element from input1 (since y4=1 and y3 is handled by scalar_broadcast_f). But in the code, after each scalar_broadcast_f call (which is per i2), input1_data_ptr is incremented by 1. That would mean that for each i2 iteration, a new input1 element is used. But according to the broadcast pattern, input1 should be broadcast along y3, which in this case, since y4=1, perhaps the y3 dimension is part of the broadcast. Wait, the comment says:
-"In the fivefold pattern, y0, y2 and y4 are not broadcast, and so shared between input shapes. y3 for input 1 is always broadcast, and so the dimension there is 1, whereas optionally y1 might be broadcast for input 2. Put another way, input1.shape.FlatSize = y0 * y1 * y2 * y4, input2.shape.FlatSize = y0 * y2 * y3 * y4."
-So input1's shape is [y0, y1, y2, y4], and input2's shape is [y0, y2, y3, y4]. The broadcasted shape is [y0, y1, y2, y3, y4], but since y3 is broadcast for input1 (so input1's y3 dimension is 1), and y1 may be broadcast for input2.
-In the special case where y4 == 1, the code is handling the inner loop differently. For input1, each element in the y2 dimension (i2 loop) would correspond to a single element (since y4=1), and this element is broadcast across y3 elements (since input1's y3 dimension is 1, so it's broadcasted to match input2's y3 dimension). Therefore, in the scalar_broadcast_f function, the input1 element should be the same for all y3 elements. However, in the code, after each scalar_broadcast_f call (which processes y3 elements), the input1_data_ptr is incremented by 1. That would mean that each subsequent scalar_broadcast_f call uses the next element in input1_data, which would not be a broadcast but a strided access. This is a mistake.
-For example, suppose y3 is 5. Then scalar_broadcast_f would process 5 elements, using the same input1 element. But the code increments input1_data_ptr by 1 after that, so the next scalar_broadcast_f would use the next element. This would only be correct if the input1 has a dimension of y3 in that position, which it shouldn't because according to the broadcast pattern, input1's y3 dimension is 1 (since it's broadcasted). Therefore, the code is incorrectly advancing the input1_data_ptr by 1 for each i2 iteration, leading to accessing out of bounds if the input1_data doesn't have enough elements.
-Wait, but according to the input1.shape.FlatSize = y0 * y1 * y2 * y4. Since y4 is 1 in this case, the flat size is y0 * y1 * y2. The loops are over i0 (y0), i1 (y1), i2 (y2). So for each i0, i1, i2, there should be exactly one element in input1. Therefore, the total number of elements in input1_data should be y0 * y1 * y2. However, in the code, for each i2 iteration, input1_data_ptr is incremented by 1. Since the loop over i2 runs y2 times, and for each i0 and i1, the total number of increments would be y0 * y1 * y2, which matches the input1's flat size. So in this case, the code is correct. Because each i2 iteration corresponds to one element in input1. But wait, how does that align with the broadcasting?
-Wait, perhaps I'm misunderstanding the dimensions. Let's re-express the shapes. The broadcasted output shape is [y0, y1, y2, y3, y4]. Input1 has shape [y0, y1, y2, y4], and input2 has shape [y0, y2, y3, y4]. So when broadcasting, input1 is broadcasted along the y3 dimension (since it's missing in input1's shape), and input2 is broadcasted along the y1 dimension.
-In the special case where y4 == 1, the code is handling the inner loop (which would have been y4 elements) as a single element. So for each element in the output, which has dimensions y0, y1, y2, y3, 1, the code processes them.
-In the general case (y4 &gt; 1), the innermost loop (i3) processes y4 elements at a time. For each i3, the same input1_data_ptr is used (since input1 is broadcast along y3), and input2_data_ptr is advanced by y4 each time. Then, after processing all i3 (y3 times), input1_data_ptr is advanced by y4. So for each i2 iteration, input1_data_ptr moves forward by y4 * y3? No, wait: the loop over i3 runs y3 times, but input1_data_ptr is only advanced once after the loop. So for each i2 iteration, input1_data_ptr is advanced by y4. Because the loop over i3 doesn't change input1_data_ptr during the loop. So for each i2, the code processes y3 * y4 elements of input1, but the pointer is advanced by y4. That would imply that the same y4 elements are used for each i3 iteration, which is correct because input1 is broadcast along y3. So each i3 iteration uses the same y4 elements from input1, repeated y3 times.
-In the special case (y4 == 1), the code uses scalar_broadcast_f, which takes a single element from input1 (since y4=1) and broadcasts it across y3 elements. Therefore, in this case, for each i2 iteration, the code should use the same input1 element for all y3 elements. However, in the code, after the scalar_broadcast_f call, input1_data_ptr is incremented by 1. That would mean that each i2 iteration uses a new input1 element, which would be correct if the input1 has a dimension of y2 in that position. But according to the input1's shape, which is [y0, y1, y2, y4], with y4=1, the total elements are y0*y1*y2. The loops are over i0 (y0), i1 (y1), i2 (y2). So each i2 iteration corresponds to one element in input1. Therefore, incrementing input1_data_ptr by 1 after each i2 iteration is correct. Because for each i2, you have one element in input1, which is broadcast across y3 elements (handled by scalar_broadcast_f). Therefore, the code is correct here.
-Wait, that makes sense. Because in the special case, each i2 iteration processes one element from input1 (since y4=1), and that element is broadcast across y3 elements in the output. So the scalar_broadcast_f function would take that single element and replicate it y3 times. Therefore, after processing that i2 iteration, the input1_data_ptr is advanced by 1 to point to the next element for the next i2 iteration. So this is correct.
-So in this case, the code seems to handle the pointers correctly. Then, where could a vulnerability be?
-Another thing to check is the use of the variables y0, y1, y2, y3, y4. These are derived from params.broadcast_shape[0] to [4]. If these values are not properly validated, they could be very large, leading to integer overflows when multiplied together, or causing the loops to run for a very long time (denial of service). However, in practice, such code would typically have checks on the input shapes before entering this function.
-Another possible issue is the use of the elementwise_f and scalar_broadcast_f function pointers. If these functions are not properly validated, they could be pointing to malicious code, but that's more of a concern in other contexts, like if this code is part of a JIT compiler or something. But assuming that these functions are part of the framework and properly controlled, this might not be an issue.
-Looking at the code again, in the general case, the input2_data_ptr is set to input2_data_reset at the start of the i1 loop. Then, for each i2 and i3, it's advanced. After the i1 loop, input2_data_reset is updated to input2_data_ptr. This seems to be handling the broadcasting correctly for input2.
-Another thing to check is whether the loops correctly handle all dimensions. For example, in the general case, the loops are i0, i1, i2, i3, and the innermost elementwise_f handles y4 elements. The total number of elements processed should be y0 * y1 * y2 * y3 * y4, which matches the output shape. Similarly for the special case.
-But what if any of the y0, y1, y2, y3, y4 are zero? The loops would not run, so no problem. Negative values would be a problem, but again, assuming the shapes are validated.
-Another possible issue is the use of the variables without checking their validity. For example, if y3 is zero, but the code still calls scalar_broadcast_f with y3=0. But that function should handle that.
-Wait, but in the special case code, there's a condition:
-} else if (input1_data_ptr != nullptr) {
-So if input1_data_ptr is null, this code path isn't taken. But how is input1_data_ptr determined? It's either unswitched_input1_data or unswitched_input2_data, depending on use_unswitched. If those inputs are null, then this could lead to a null pointer dereference. However, the code checks if input1_data_ptr is not null before entering the special case. But in the general case, there's no such check. So if input1_data or input2_data is null, and the code enters the general case, it would dereference a null pointer.
-Ah, this could be a vulnerability. Let's see:
-The function parameters include unswitched_input1_data and unswitched_input2_data, which are const T*. These could be null pointers if the input shapes are empty or invalid. However, the code does not check if these pointers are null before dereferencing them.
-In the general case, the code uses input1_data_ptr and input2_data_ptr, which are set based on use_unswitched. If either of the input data pointers is null, then dereferencing them would cause a crash.
-For example, if unswitched_input1_data is null and use_unswitched is true, then input1_data_ptr would be null. Then, in the general case, when the code does input1_data_ptr += y4; or passes it to elementwise_f, which likely dereferences it, this would be a null pointer dereference.
-Similarly, in the special case, the code checks if input1_data_ptr is not null before proceeding. But in the general case, there's no such check.
-So this is a potential vulnerability. If an attacker can control the input data pointers to be null, they could cause a null pointer dereference, leading to a crash (denial of service) or potentially other exploits depending on the environment.
-But wait, in the special case, the code checks if (input1_data_ptr != nullptr) before entering the else block. However, in the general case (the first if block), there's no such check. So if the code enters the general case with input1_data_ptr or input2_data_ptr being null, then the code would dereference null pointers.
-Therefore, this is a vulnerability. The code does not check for null pointers in the general case.
-But how likely is this to happen? It depends on how the function is called. If the function is part of a larger framework that ensures that input data pointers are valid (non-null) when the shapes are non-empty, then this might not be an issue. However, if the framework allows empty tensors (with zero-sized shapes) but non-null data pointers, or if there's a way to have a null pointer passed in, then this could be a problem.
-In C++, dereferencing a null pointer is undefined behavior, which can lead to crashes or security vulnerabilities.
-Therefore, the code is vulnerable because it does not check for null pointers in the general case. The special case checks for input1_data_ptr != nullptr, but the general case does not.
-Another thing to check: in the general case, the code uses input2_data_reset, which is initialized to input2_data. If input2_data is null, then input2_data_reset is null, and in the loop, input2_data_ptr is set to input2_data_reset (null), and then in elementwise_f, it would be dereferenced.
-So yes, this is a vulnerability. The code should check that input1_data and input2_data are not null before proceeding, especially in the general case.
-Therefore, the answer should be YES, vulnerability detected.
-&lt;/think&gt;
-(1) YES: Vulnerability detected.
+          <t>(1) YES: Vulnerability detected.
 **Step-by-Step Explanation:**
 1. **Null Pointer Dereference in General Case:**
    - The function uses `input1_data` and `input2_data` pointers derived from `unswitched_input1_data` and `unswitched_input2_data`. These pointers could be null if the input shapes are invalid or empty.
@@ -2931,123 +2806,7 @@
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>We are analyzing the provided code for potential vulnerabilities. The function `qf_fill_buffer` is part of a Vim-like editor (likely the quickfix feature). We are to determine if there is a vulnerability.
-Let's break down the code step by step and look for common security issues such as:
-- Buffer overflows
-- Use-after-free
-- Integer overflows
-- Format string vulnerabilities
-- Uninitialized variables
-- Race conditions (but note: static analysis, so we focus on code structure)
-- Other memory corruption issues
-We'll go through the code:
-1. **Initialization and Setup**:
-   - `old_KeyTyped` is saved (a global variable, but we don't know its type, but it's likely an integer).
-   - `qftf_list` and `qftf_li` are initialized to NULL.
-2. **Handling `old_last == NULL`**:
-   - If `old_last` is NULL and `buf` is not the current buffer, it calls `internal_error` and returns. This is a safety check.
-3. **Deleting existing lines**:
-   - If `old_last` is NULL and `buf` is not the current buffer, it returns (already handled above). Otherwise, it deletes all existing lines in the buffer (by deleting line 1 until the buffer is empty). This is safe because it's using `ml_delete` which is a known safe function for the buffer.
-4. **Checking if there is anything to display**:
-   - If `qfl` is not NULL, then it proceeds.
-5. **Setting up for adding lines**:
-   - `dirname` is set to empty (a buffer of MAXPATHL, which is a fixed size, so no overflow here).
-   - `invalid_val` is set to FALSE.
-   - `prev_bufnr` is set to -1.
-6. **Determining the starting point for adding lines**:
-   - If `old_last` is NULL, then `qfp` starts at `qfl-&gt;qf_start` and `lnum` is 0.
-   - Otherwise, it starts from `old_last-&gt;qf_next` (or `old_last` if `old_last-&gt;qf_next` is NULL) and `lnum` is set to the current line count of the buffer.
-7. **Calling a user-defined function**:
-   - `qftf_list = call_qftf_func(...)` - This function is called with parameters including `qf_winid` and `lnum+1`. The return value is a list (or NULL). We don't know what `call_qftf_func` does, but it's a function that the user can define (via Vim script). However, note that the function is called with `qf_winid` (a window ID) and `lnum+1` (a line number). The function returns a list of strings (or something that can be converted to a string) for the lines to display.
-8. **Processing the list**:
-   - `qftf_li` is set to the first item of the list (if the list is not NULL).
-   - Then, a loop runs from `lnum` to `qfl-&gt;qf_count` (the total number of lines in the quickfix list).
-9. **Processing each line**:
-   - It checks if `qftf_li` is not NULL and `invalid_val` is false. Then it gets a string from the list item (using `tv_get_string_chk`). If that returns NULL, it sets `invalid_val` to TRUE (so that the rest of the list is ignored and default is used).
-   - Then it calls `qf_buf_add_line` to add a line to the buffer. This function takes:
-        - `buf`: the buffer to add to
-        - `lnum`: the line number to add at (starting from 0, but note: the buffer lines are 1-indexed? Actually, the function `ml_delete` uses 1-indexed, so likely the buffer is 1-indexed. However, note that `lnum` is being incremented and used as the line number to add at. The function `qf_buf_add_line` is not provided, but we have to assume it's safe. However, note that `lnum` is being incremented and used as the line number for the new line. The buffer is being built from scratch (if `old_last` is NULL) so the current line count is `lnum` (which starts at 0 or the current count) and then we are adding lines one by one.
-10. **After the loop**:
-    - If `old_last` is NULL, it deletes the empty line at the end (which was added by the loop? Actually, the loop adds lines until `qfl-&gt;qf_count`, and then if `old_last` is NULL, it deletes the line at `lnum+1` (which would be the next line after the last added line). This is safe because the buffer has exactly `lnum` lines (if we started at 0 and added `qfl-&gt;qf_count` lines, then `lnum` becomes `qfl-&gt;qf_count`). Then deleting line `lnum+1` (which is beyond the current last line) would be a no-op? Actually, the buffer has `lnum` lines (so the last line is `lnum`). Then `lnum+1` is the next line, which doesn't exist. But note: the loop condition is `lnum &lt; qfl-&gt;qf_count`, so when the loop ends, `lnum` is equal to `qfl-&gt;qf_count` (if it broke on the condition). Then `lnum+1` is `qfl-&gt;qf_count+1`, which is beyond the current buffer (which has `qfl-&gt;qf_count` lines). So `ml_delete(lnum+1)` would delete a line that doesn't exist? Actually, `ml_delete` deletes a line by number. If the line number is beyond the current number of lines, it does nothing? We don't know, but it's safe because it's a deletion of a non-existent line.
-11. **Setting the filetype**:
-    - If `old_last` is NULL, it sets the filetype to "qf", and applies autocommands. This is safe.
-12. **Restoring `KeyTyped`**:
-    - Restores the saved `KeyTyped`.
-Now, let's look for vulnerabilities:
-- **Buffer overflows**: 
-  - The `dirname` buffer is of fixed size `MAXPATHL` and is set to NUL (empty) at the beginning. Then it's passed to `qf_buf_add_line`. We don't know what `qf_buf_add_line` does with `dirname`, but it's a fixed-size buffer and we are not writing to it beyond its size. So no overflow here.
-- **Integer overflows**:
-  - The loop condition: `lnum &lt; qfl-&gt;qf_count`. `lnum` starts at 0 (or the current line count) and is incremented until it reaches `qfl-&gt;qf_count`. The variable `qfl-&gt;qf_count` is the total number of lines in the quickfix list. We don't know the type of `qf_count`, but it's likely an integer. However, note that `lnum` is incremented by one each time and the loop condition is `lnum &lt; qfl-&gt;qf_count`. So the maximum value of `lnum` is `qfl-&gt;qf_count - 1`. Then we do `lnum++` and then `lnum` becomes `qfl-&gt;qf_count` and the loop condition fails. So no integer overflow in the loop.
-  - Also, note that `qfl-&gt;qf_count` is used as the upper bound. We don't know if it's a large number, but the buffer can only hold so many lines. However, the function `ml_delete` and `qf_buf_add_line` are designed to handle the buffer, so we assume they are safe.
-- **Use-after-free**:
-  - We don't see any free operations on the `qfl` structure. The `qfl` is a pointer to a `qf_list_T` which is a linked list. The function uses `qfp` to traverse the list. There is no freeing of the list in this function, so no use-after-free.
-- **Format string vulnerability**:
-  - We don't see any `printf`-like functions that take a format string from user input. The only string operations are with `dirname` (which is set to empty) and the string from `tv_get_string_chk` (which is a string from the user-defined function). But note: `tv_get_string_chk` returns a string that is then passed to `qf_buf_add_line`. We don't know what `qf_buf_add_line` does, but it's unlikely to use it as a format string. Also, the string is not passed to a function that uses it as a format string (like `printf`). So no.
-- **Uninitialized variables**:
-  - `dirname` is initialized to NUL (so it's safe). 
-  - `invalid_val` is set to FALSE.
-  - `prev_bufnr` is set to -1.
-  - `qftf_list` and `qftf_li` are set to NULL initially.
-- **Other issues**:
-  - The function `call_qftf_func` is called with `qf_winid` and `lnum+1`. We don't know what this function does, but it's a user-defined function (via Vim script). However, the vulnerability we are looking for is in the C code, not in the script. The C code is safe as long as it handles the return value correctly. The code checks for NULL and for invalid string (by setting `invalid_val` and then ignoring the rest). So it's safe.
-  - The function `qf_buf_add_line` is called with `qftf_str` which might be NULL (if `tv_get_string_chk` returns NULL, then `invalid_val` is set and the rest of the list is ignored, and then `qftf_str` is NULL). The function `qf_buf_add_line` should handle a NULL string (probably by using a default). We don't have the code for that, but the function is called with `qftf_str` and the function is expected to handle it. The code does not crash because it checks for NULL and then uses the default (by setting `invalid_val` and then the rest of the loop uses the default). So it's safe.
-  - The `qf_buf_add_line` function is called with `lnum` (which is the current line number to add at). The buffer is being built from scratch (if `old_last` is NULL) so the current line count is `lnum` (which is 0 at the start). Then we add a line at `lnum` (which is 0) but note: the buffer is 1-indexed? Actually, the `ml_delete` function uses 1-indexed, so the buffer lines are 1-indexed. However, the function `qf_buf_add_line` is not provided, but we can assume it uses the same indexing. The function `ml_delete` deletes line 1, so the buffer is 1-indexed. Therefore, when adding a line at `lnum=0`, that would be an invalid line number? But note: the function `qf_buf_add_line` is called with `lnum` (which is the current line count, meaning the next line to add is at `lnum+1`? Actually, the function `qf_buf_add_line` is called with `lnum` as the line number to add at. In the context of the buffer, if the buffer currently has `lnum` lines, then the next line to add is at `lnum+1`? But the function is called with `lnum` (which is the current count) and then it adds a line at that position? Actually, the function `qf_buf_add_line` is likely designed to add a line at the specified line number (so if the buffer has 0 lines, then adding at line 0 would be invalid). However, note that the code sets `lnum` to 0 when `old_last` is NULL. Then it calls `qf_buf_add_line` with `lnum=0`. This might be a bug, but it's not a vulnerability (it's a bug that might cause a crash, but we are looking for security vulnerabilities). However, the problem says "vulnerability", which typically means a security flaw that can be exploited (like arbitrary code execution, information leak, etc.). A crash is a vulnerability (denial of service) but it's not a typical security vulnerability. But note: the problem says "vulnerability" in the context of security, so we are to look for security issues.
-  However, let's check: the function `qf_buf_add_line` is called with `lnum` (which is 0) and the buffer is empty. The function `ml_append` (which is likely used inside `qf_buf_add_line`) would expect a line number that is at least 1. So if `qf_buf_add_line` uses `ml_append` with `lnum` (which is 0) as the line number, then it would be invalid. But note: the function `ml_append` in Vim is called with a line number (1-indexed) and it appends at the end if the line number is beyond the current count. However, the function `ml_append` in Vim actually takes a line number and inserts before that line. So if you want to append, you use `ml_append` with `lnum = curbuf-&gt;b_ml.ml_line_count + 1`. But in our case, the function `qf_buf_add_line` is called with `lnum` (which is the current line count) and then it adds a line at that position? Actually, the function `qf_buf_add_line` is not provided, so we have to assume it's implemented correctly. But note: the code that calls it is setting `lnum` to the current line count (which is the number of lines already in the buffer). Then it adds a line at `lnum` (which would be the next line, so it should be `lnum+1`). However, the function `qf_buf_add_line` might be designed to add at the current line count (meaning the next line). So it's likely that the function uses `lnum+1` internally? We don't know.
-  But note: the code does:
-      if (qf_buf_add_line(buf, lnum, ...) == FAIL)
-          break;
-  And then it does `++lnum` and then `qfp = qfp-&gt;qf_next;`.
-  So the first call: `lnum=0` (if `old_last` is NULL) -&gt; adds a line at position 0? That would be invalid. However, the buffer is empty, so the current line count is 0. The function `qf_buf_add_line` should probably be adding at the end, so it should use `lnum+1` (which is 1). But the function is called with `lnum` (0). This might be a bug, but it's not a security vulnerability. It's a bug that might cause a crash (if the function doesn't handle line 0 correctly). However, the problem is about security vulnerabilities, and a crash is a vulnerability (denial of service) but it's not a typical one we are looking for. Moreover, the problem says "vulnerability" in the context of security, and we are to decide if it's vulnerable (YES) or not (NO). But note: the problem does not specify the type of vulnerability.
-  However, let's look at the code again: the function `qf_buf_add_line` is called with `lnum` (which is the current line count). In the buffer, the current line count is the number of lines. The next line to add should be at `lnum+1` (1-indexed). So the function should be called with `lnum+1`? But it's called with `lnum`. This is a bug, but it's not a security vulnerability per se. It's a bug that might cause a crash, but the problem is about security.
-  But note: the code also has a similar call when `old_last` is not NULL: `lnum` is set to `buf-&gt;b_ml.ml_line_count` (the current line count). Then it adds a line at `lnum` (which would be the next line, so it should be `lnum+1`). So the same issue.
-  However, the function `qf_buf_add_line` might be designed to take the line number as the position to insert (so 0 would be invalid, but 1 would be the first line). But the buffer is empty, so the first line should be inserted at 1. Therefore, the call with `lnum=0` is wrong. But the function `qf_buf_add_line` might handle it by using `lnum+1` internally? We don't know. But note: the code that calls `qf_buf_add_line` is written by the author, so it's likely that the function expects the line number to be the position (1-indexed) and the current line count is the number of lines, so the next line is at `current_line_count + 1`. Therefore, the call should be with `lnum+1`? But it's called with `lnum`.
-  However, the code does:
-      lnum = buf-&gt;b_ml.ml_line_count;   // for the non-NULL old_last case
-  Then it calls `qf_buf_add_line(buf, lnum, ...)`. But the buffer has `lnum` lines, so the next line should be at `lnum+1`. So the call should be with `lnum+1`. But it's called with `lnum`. This is a bug.
-  But note: the function `qf_buf_add_line` might be designed to take the line number as the index (0-indexed) and then convert it to 1-indexed? We don't know. However, the problem is that we are to analyze the code for vulnerabilities, and this bug might lead to a crash (if the function doesn't handle 0 correctly). But is it a security vulnerability? It's a bug that could be exploited to cause a crash (denial of service), but it's not a typical security vulnerability (like arbitrary code execution). However, the problem does not specify, so we have to consider it.
-  But note: the problem says "vulnerability" in the context of security, and in the security field, a crash is a vulnerability (it's a denial of service). However, the problem might be expecting a more severe vulnerability.
-  Let's look for something else.
-- **User-controlled input**:
-  - The function `call_qftf_func` is called with `qf_winid` and `lnum+1`. The `qf_winid` is a window ID (which is controlled by the user, but it's an integer). The `lnum+1` is a line number (which is controlled by the number of lines in the buffer, which is controlled by the user via the quickfix list). But the function `call_qftf_func` is a function that the user can define (via Vim script). The user can define a function that returns a very long string? But note: the string is then passed to `tv_get_string_chk` and then to `qf_buf_add_line`. The `qf_buf_add_line` function is responsible for handling the string. It's unlikely to cause a buffer overflow because the string is being added to the buffer (which is a line in the buffer, and the buffer can grow). However, the string might be very long, but that would just make the buffer large, not cause a vulnerability.
-  - The `dirname` buffer is set to empty and then passed to `qf_buf_add_line`. The `dirname` is set to NUL at the beginning, so it's safe.
-  - The `qftf_str` is obtained from the user-defined function. The user can return a string of arbitrary length. But the function `qf_buf_add_line` is expected to handle it (by adding it as a line). The buffer can grow to accommodate the string, so no overflow.
-  - The only potential issue is the line number passed to `qf_buf_add_line` (the `lnum` argument) being 0 when the buffer is empty. But as discussed, that might cause a crash, but it's not a security vulnerability in the sense of arbitrary code execution.
-  However, note: the function `qf_buf_add_line` might be implemented in a way that uses `lnum` as an index without checking. For example, if it does:
-        ml_append(lnum, ...);
-  and `lnum` is 0, then `ml_append` might crash because it expects a line number &gt;= 1.
-  But the `ml_append` function in Vim (from the source) actually does:
-        if (lnum &lt;= 0)
-            lnum = 1;
-        else if (lnum &gt; curbuf-&gt;b_ml.ml_line_count + 1)
-            lnum = curbuf-&gt;b_ml.ml_line_count + 1;
-  So it normalizes the line number. Therefore, passing 0 would be converted to 1. So it's safe.
-  Therefore, the bug we thought of (passing 0) is actually handled by the underlying `ml_append` (or similar) function.
-  So the code is safe in that regard.
-- **Other potential issues**:
-  - The function `call_qftf_func` might be called with a very large `lnum+1`? But `lnum` is the current line count (which is at most the number of lines in the buffer, which is limited by the system). And `qfl-&gt;qf_count` is the total number of lines in the quickfix list, which is also limited. So no integer overflow in the arguments.
-  - The function `qf_buf_add_line` might have a bug, but we don't have its code. We are only to analyze the provided code.
-After reviewing, I don't see any obvious security vulnerability (like buffer overflow, use-after-free, format string, etc.) in the provided code.
-However, note that the code does:
-    if (old_last == NULL)
-    {
-        // delete all existing lines
-        while ((curbuf-&gt;b_ml.ml_flags &amp; ML_EMPTY) == 0)
-            (void)ml_delete((linenr_T)1);
-    }
-This deletes the entire buffer. But note: `ml_delete` is called with line 1. If the buffer is empty, then `ml_delete(1)` would do nothing (because the buffer has no line 1). So it's safe.
-Also, note that the function `ml_delete` is called in a loop until the buffer is empty. This is safe.
-Another point: the function `qf_buf_add_line` is called with `qftf_str` which might be NULL (if the user-defined function returns a non-string). But the code sets `invalid_val` to TRUE and then ignores the rest of the list. So it's safe.
-Therefore, I conclude that there is no vulnerability.
-But let's double-check for a specific vulnerability: the "qf_buf_add_line" function might be vulnerable to a buffer overflow if it copies the string without checking the length? However, the string is being added to a buffer line, and the buffer line can grow. The function `ml_append` (which is likely used) uses `vim_strsave` to copy the string, so it's safe.
-So the answer should be NO.
-However, note that the problem says "static program analysis", and we are to decide based on the code provided.
-Final decision: NO.
-But wait: there is one more thing. The function `call_qftf_func` is called with `qf_winid` and `(long)(lnum + 1)`. The `lnum` is an integer that might be large, but it's cast to `long`. This is safe because `lnum` is a line number (which is not huge). But note: the `qf_winid` is an integer (window ID) and it's passed as a `long`? But the function `call_qftf_func` expects a `long`? We don't know, but it's a safe cast.
-Also, note that the function `call_qftf_func` is called with `qf_winid` (which is a window ID) and `lnum+1` (a line number). The user-defined function might do anything, but the C code is safe.
-Therefore, I think there is no vulnerability.
-Answer: NO
-&lt;/think&gt;
-After a thorough static analysis of the provided code, I have identified no security vulnerabilities. Here's the step-by-step reasoning:
+          <t>After a thorough static analysis of the provided code, I have identified no security vulnerabilities. Here's the step-by-step reasoning:
 1. **Buffer Handling**:
    - `dirname` is a fixed-size buffer (`MAXPATHL`) initialized to `NUL` (empty). It's only used as a parameter to `qf_buf_add_line`, which safely handles string input (no overflow risk).
    - `qftf_str` (from user-defined function) is validated via `tv_get_string_chk` before use. If invalid, `invalid_val` is set to skip further processing (no use-after-free or invalid string handling).
@@ -3480,130 +3239,7 @@
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>We are analyzing the provided code for potential vulnerabilities. The code is a method `Compute` of an `OpKernel` in TensorFlow (or a similar framework). We are to check for security vulnerabilities, particularly in the context of static program analysis.
-Key points to consider:
-1. **Input Validation**: The code checks for various conditions on the inputs (like shape, dimensions, etc.) using `OP_REQUIRES` which will fail the operation if the condition is not met. This is a good practice to prevent invalid inputs from causing issues.
-2. **Array Bounds and Indexing**: We need to check if there are any off-by-one errors, buffer overflows, or out-of-bounds accesses.
-3. **Memory Allocation**: The code uses `ctx-&gt;allocate_output` to allocate memory for outputs. We must check if the allocation sizes are correctly computed and if they are within safe bounds.
-4. **Tensor Dimensions and Shapes**: The code uses tensor dimensions and shapes to index and access data. We must ensure that the indices used are within the bounds of the tensors.
-Let's break down the code step by step:
-- `const Tensor&amp; gradient = ctx-&gt;input(0);`
-- `const Tensor&amp; input = ctx-&gt;input(1);`
-- `Tensor* input_backprop = nullptr;`
-- `OP_REQUIRES_OK(ctx, ctx-&gt;allocate_output(0, input.shape(), &amp;input_backprop));` 
-  - This allocates an output tensor of the same shape as `input`. Since `input.shape()` is used, the allocation is safe in terms of the tensor's own shape.
-- `OP_REQUIRES(ctx, axis_ &gt;= -1, ...);` 
-  - Checks that `axis_` is at least -1.
-- `OP_REQUIRES(ctx, (axis_ == -1 || axis_ &lt; input.shape().dims()), ...);`
-  - Checks that if `axis_` is not -1, then it must be less than the number of dimensions of `input`. This is safe because `axis_` is compared to `input.shape().dims()` (which is the number of dimensions) and `axis_` is an integer.
-- `OP_REQUIRES(ctx, input.IsSameSize(gradient), ...);`
-  - Ensures that `gradient` and `input` have the same size (i.e., same number of elements). This is important for the subsequent operations.
-- `const int depth = (axis_ == -1) ? 1 : input.dim_size(axis_);`
-  - If `axis_` is -1, `depth` is set to 1. Otherwise, it's set to the size of the `axis_` dimension of `input`.
-  - Note: `axis_` is checked to be in the valid range (either -1 or between 0 and `input.shape().dims()-1`), so `input.dim_size(axis_)` is safe.
-- Then, it gets `input_min_tensor` and `input_max_tensor` from inputs 2 and 3.
-- Checks for `input_min_tensor` and `input_max_tensor` dimensions: must be 0 or 1. This is safe.
-- If `axis_ != -1`, it checks that the first dimension of `input_min_tensor` and `input_max_tensor` equals `depth` (which is the size of the axis dimension of `input`). This is safe because `depth` is computed from `input` and the axis is valid.
-- Then, it sets `min_max_shape` to the shape of `input_min_tensor` (which is either a scalar or a 1D tensor) and allocates outputs for `input_min_backprop` and `input_max_backprop` with that shape.
-- The code then branches on `axis_`:
-  **Case 1: axis_ == -1**
-    - Checks that `input_min_tensor` and `input_max_tensor` are scalars (using `TensorShapeUtils::IsScalar`). This is safe because we already checked the dimensions (0 or 1) and then for axis_=-1 we require scalar (which is dimension 0? Actually, note: a scalar has 0 dimensions, but the code checks for scalar with `IsScalar`). The `IsScalar` function in TensorFlow typically checks for 0 dimensions.
-    - Then it calls a functor that uses:
-        - `input_min_tensor.scalar&lt;T&gt;()` -&gt; which gets the scalar value. Since it's a scalar, this is safe.
-        - Similarly for `input_max_tensor.scalar&lt;T&gt;()`.
-    - The functor is called with:
-        - `gradient.template flat&lt;T&gt;()` -&gt; flat tensor (all elements in one dimension) of the gradient tensor.
-        - `input.template flat&lt;T&gt;()` -&gt; same for input.
-        - `input_backprop-&gt;template flat&lt;T&gt;()` -&gt; same for the output.
-        - `input_min_backprop-&gt;template scalar&lt;T&gt;()` and `input_max_backprop-&gt;template scalar&lt;T&gt;()` -&gt; which are scalars.
-    - Since the tensors are flat (all elements) and the scalar access is safe (because we checked they are scalars), there are no out-of-bounds issues.
-  **Case 2: axis_ != -1**
-    - The functor `QuantizeAndDequantizePerChannelGradientFunctor` is called with:
-        - `gradient.template flat_inner_outer_dims&lt;T, 3&gt;(axis_ - 1)`
-        - `input.template flat_inner_outer_dims&lt;T, 3&gt;(axis_ - 1)`
-        - `&amp;input_min_tensor` (a reference to the tensor, not a scalar)
-        - `&amp;input_max_tensor`
-        - `input_backprop-&gt;template flat_inner_outer_dims&lt;T, 3&gt;(axis_ - 1)`
-        - `input_min_backprop-&gt;template flat&lt;T&gt;()` (which is a flat tensor of the min_backprop output, which is the same shape as input_min_tensor, so it's safe)
-        - `input_max_backprop-&gt;template flat&lt;T&gt;()`
-    - The `flat_inner_outer_dims` function is used to reshape the tensor for the given axis. The function `flat_inner_outer_dims` in Eigen (used in TensorFlow) is safe as long as the axis is within the valid range. We have already checked that `axis_` is in [0, input.shape().dims()-1] (because we have `axis_ != -1` and `axis_ &lt; input.shape().dims()`). Note: the function uses `axis_ - 1` as the axis for the reshape. But note: the axis we are using in the tensor is 0-indexed, and the `axis_` we have is the same as the one passed (which is 0-indexed for the tensor). However, the code subtracts 1. Why?
-      Let me clarify: 
-        - The tensor has `input.shape().dims()` dimensions.
-        - The `axis_` we have is the axis index (0-indexed) for the tensor. But note: the condition `axis_ &lt; input.shape().dims()` ensures that `axis_` is in [0, input.shape().dims()-1]. Then we do `axis_ - 1` in the call to `flat_inner_outer_dims`.
-      This would be a problem if `axis_` is 0, because then we are using `-1` as the axis. However, note the condition: `axis_` is at least 0 (because we are in the branch `axis_ != -1` and we have `axis_ &gt;= -1` and then we checked `axis_ &lt; input.shape().dims()`). But note: the condition `axis_ &gt;= -1` and then `axis_ != -1` implies `axis_ &gt;= 0`. So `axis_` is at least 0. Then `axis_ - 1` would be at least -1.
-      However, the `flat_inner_outer_dims` function in Eigen (and in TensorFlow) expects the axis to be non-negative? Actually, the function `flat_inner_outer_dims` in TensorFlow's Eigen wrappers is defined for a given axis (which is the dimension index to split). The axis index must be in the range [0, num_dims-1]. But here we are passing `axis_ - 1` which for `axis_ = 0` becomes -1. This is invalid.
-      Let's check the condition again: 
-        - The condition `OP_REQUIRES(ctx, (axis_ == -1 || axis_ &lt; input.shape().dims()), ...)` ensures that if `axis_` is not -1, then `axis_` is less than the number of dimensions. But note: the condition does not require `axis_` to be non-negative? Actually, the condition `axis_ &gt;= -1` and then `axis_ &lt; input.shape().dims()` for non -1, but note: `axis_` could be negative? The condition `axis_ &gt;= -1` allows -1 and non-negative. However, the condition for non -1 is `axis_ &lt; input.shape().dims()`, but it does not say `axis_ &gt;= 0`. So `axis_` could be negative (but not -1) and then we have a problem.
-      But wait: the condition `axis_ &gt;= -1` and then the next condition: `axis_ == -1 || axis_ &lt; input.shape().dims()`. This condition does not require `axis_` to be non-negative. So if `axis_` is -2, it would pass the first condition (&gt;= -1? no, -2 &lt; -1) so it would fail the first condition. Actually, the first condition is `axis_ &gt;= -1`, so `axis_` must be at least -1. Therefore, the only negative value allowed is -1. So in the branch `axis_ != -1`, `axis_` must be &gt;=0. Therefore, `axis_` is in [0, input.shape().dims()-1]. Then `axis_ - 1` is in [-1, input.shape().dims()-2]. But note: when `axis_` is 0, `axis_ - 1` is -1, which is invalid for the `flat_inner_outer_dims` function.
-      This is a bug. However, note that the condition for the axis in the non -1 branch also has a check: `axis_ != -1` and then we have the condition that `axis_` is less than the number of dimensions. But the function `flat_inner_outer_dims` expects a non-negative axis. So when `axis_` is 0, we are passing -1 to `flat_inner_outer_dims`, which is invalid.
-      But wait: the code in the non -1 branch uses `axis_ - 1` as the axis for the reshape. Why? Let me see the context. The `flat_inner_outer_dims` function in TensorFlow (for example, in `eigen_tensor.h`) is defined as:
-        template &lt;typename T, int N&gt;
-        Eigen::TensorMap&lt;Eigen::Tensor&lt;T, N, Eigen::RowMajor&gt;&gt; flat_inner_outer_dims(int axis) const;
-      The `axis` parameter is the dimension index to split. The tensor is split into two parts: the inner dimensions (from 0 to axis-1) and the outer dimensions (from axis to the end). The axis must be in [0, num_dims-1]. So if we pass -1, it's invalid.
-      Therefore, the code has a bug: when `axis_` is 0, we are passing -1 to `flat_inner_outer_dims`, which is invalid and will cause a crash (or undefined behavior).
-      However, note: the condition for the axis in the non -1 branch does not prevent `axis_` from being 0. And the code does not check for `axis_` being 0. So this is a vulnerability? Actually, it's a bug that might cause a crash, but is it a security vulnerability? In the context of a kernel, a crash might be a denial of service (DoS) vulnerability. But note: the input `axis_` is provided by the user (or the graph). The kernel is designed to fail with an error if the axis is invalid. However, the current condition does not catch the case when `axis_` is 0? Actually, the condition `axis_ &lt; input.shape().dims()` allows `axis_` to be 0 (since 0 &lt; input.shape().dims() is true if input has at least 1 dimension). So the condition passes, but then the code uses `axis_ - 1` which is -1 and causes a crash.
-      But note: the condition `axis_ &gt;= -1` and `axis_ &lt; input.shape().dims()` for non -1 does not require `axis_` to be at least 0? Actually, it does: because `axis_` is an integer and the condition `axis_ &gt;= -1` and `axis_ != -1` implies `axis_ &gt;= 0`. So `axis_` is at least 0. But the problem is that the code subtracts 1 without checking if `axis_` is 0.
-      Therefore, the code has a bug that will cause a crash when `axis_` is 0. This is a vulnerability because it can be triggered by an invalid input (axis=0) and cause the process to crash (DoS).
-      However, note: the condition for the axis in the non -1 branch also has a check for the size of the min and max tensors. But that doesn't prevent the crash in the functor call.
-      But wait: the condition `OP_REQUIRES(ctx, (axis_ == -1 || axis_ &lt; input.shape().dims()), ...)` does not require `axis_` to be non-negative? Actually, it does: because `axis_` must be at least -1 (from the first condition) and then for non -1, it must be less than the number of dimensions. But note: the condition `axis_ &lt; input.shape().dims()` for non -1 does not require `axis_` to be non-negative? It doesn't, but the first condition `axis_ &gt;= -1` and the fact that we are in the non -1 branch (so `axis_ != -1`) implies `axis_ &gt;= 0`. So `axis_` is non-negative. However, the code then subtracts 1 without checking if it's zero.
-      This is a bug. But is it a vulnerability? In the context of security, a crash (DoS) is a vulnerability. However, note that the kernel is designed to fail with an error for invalid inputs. But the current condition does not catch the invalid axis for the `flat_inner_outer_dims` function. The condition we have is for the axis being in the range [0, input.shape().dims()-1] for the tensor, but the function `flat_inner_outer_dims` requires the axis to be in [0, input.shape().dims()-1] as well. However, the code is using `axis_ - 1` which is not the same as the axis we are using for the tensor.
-      Why is the code subtracting 1? It might be a mistake. The intended axis for the tensor is `axis_`, but the function `flat_inner_outer_dims` expects the axis index (0-indexed) to be the same as the tensor's axis. So if the tensor has an axis at position `axis_`, then we should pass `axis_` to `flat_inner_outer_dims`, not `axis_ - 1`.
-      Therefore, the code has a bug that will cause a crash when `axis_` is 0. This is a vulnerability because an attacker can provide an axis=0 and cause the kernel to crash.
-      However, note: the condition `axis_ &lt; input.shape().dims()` for non -1 does not prevent `axis_` from being 0. So the kernel will accept axis=0 and then crash.
-      But wait: the condition `axis_ &lt; input.shape().dims()` for non -1: if `input.shape().dims()` is 0 (i.e., the tensor has 0 dimensions), then `axis_` must be less than 0? But `axis_` is non-negative (&gt;=0) so it would fail. However, the condition `axis_ &lt; input.shape().dims()` when `input.shape().dims() == 0` would require `axis_ &lt; 0`, but `axis_` is non-negative, so it would fail. So the only way to get to the non -1 branch is if `input.shape().dims() &gt; 0` and `axis_` is in [0, input.shape().dims()-1]. Then, when `axis_` is 0, we pass -1 to `flat_inner_outer_dims`.
-      Therefore, the code is vulnerable to a crash when `axis_` is 0.
-      However, note: the condition for the axis in the non -1 branch also has a check for the min and max tensors: `input_min_tensor.dim_size(0) == depth` (where `depth = input.dim_size(axis_)`). When `axis_` is 0, `depth = input.dim_size(0)`. This check is done and if it fails, the kernel fails. But if it passes, then we proceed to the functor call and crash.
-      So the crash happens only when `axis_` is 0 and the min and max tensors have the correct size (which is `depth = input.dim_size(0)`). But the crash is still a vulnerability.
-      But note: the condition `axis_ &lt; input.shape().dims()` for non -1: if `input.shape().dims()` is 1, then `axis_` must be 0 (because 0 &lt; 1 is true, and 1 is not less than 1). So for a 1D tensor, `axis_` must be 0. Then the code will crash.
-      Therefore, the code is vulnerable to a crash when the input tensor is 1D and `axis_` is 0.
-      However, let's check the condition again: the condition `axis_ &lt; input.shape().dims()` for non -1. For a 1D tensor, `input.shape().dims() = 1`, so `axis_` must be less than 1, i.e., 0. So the kernel will accept `axis_ = 0` for a 1D tensor. Then the code does `axis_ - 1 = -1` and passes to `flat_inner_outer_dims`, which is invalid.
-      This is a clear bug that leads to a crash.
-      But note: the condition `axis_ &gt;= -1` and `axis_ &lt; input.shape().dims()` for non -1 does not prevent `axis_` from being 0. So the kernel does not reject axis=0 for a 1D tensor. It should reject it? Actually, the intended behavior might be that for a 1D tensor, axis=0 is valid, but the code has a bug in the functor call.
-      The fix would be to not subtract 1. The axis for the tensor is `axis_`, so we should pass `axis_` to `flat_inner_outer_dims`, not `axis_ - 1`.
-      Therefore, the code has a vulnerability (a crash) that can be triggered by a valid input (axis=0 for a 1D tensor) that the kernel should accept.
-      However, note: the condition for the axis in the non -1 branch does not require `axis_` to be at least 1. So the kernel is designed to accept axis=0. But the implementation has a bug.
-      So the vulnerability is present.
-      But wait: is this a security vulnerability? In the context of a machine learning framework, a crash in a kernel might be considered a vulnerability because it can be used to cause a denial of service. Therefore, it is a vulnerability.
-      However, note: the problem says "vulnerable" meaning a security vulnerability. A DoS is a security vulnerability.
-      Therefore, the answer should be YES.
-      But let's double-check: are there any other vulnerabilities?
-      Another point: the code uses `input_min_tensor.dim_size(0)` and `input_max_tensor.dim_size(0)` without checking if the tensor has at least one dimension. However, we have already checked that the tensor has dimension 0 or 1. For dimension 0 (scalar), `dim_size(0)` would be invalid (because a scalar has 0 dimensions, so `dim_size(0)` is out of bounds). But note: the condition for the non -1 branch (axis_ != -1) requires that the tensor has dimension 1 (because we check `input_min_tensor.dim_size(0) == depth`). So for the non -1 branch, the tensor must be 1D (so `dim_size(0)` is valid). For the -1 branch, we check that the tensor is scalar (so we don't use `dim_size(0)` in the -1 branch). So that part is safe.
-      The only vulnerability we found is the crash when `axis_` is 0.
-      However, note: the condition for the non -1 branch also has a check for the axis being less than the number of dimensions, but it does not check that the axis is at least 0? Actually, it does: because `axis_` is non-negative (as established). But the problem is the subtraction of 1.
-      Therefore, the code is vulnerable.
-      But note: the problem says "static program analysis". We are to decide based on the code. We found a bug that leads to a crash, which is a vulnerability.
-      However, let's see if the condition `axis_ &lt; input.shape().dims()` is sufficient to prevent the crash? It is not, because the crash happens when `axis_` is 0 (which is allowed) and then we subtract 1.
-      So the answer is YES.
-      But wait: the condition `axis_ &lt; input.shape().dims()` for non -1: the `input.shape().dims()` is the number of dimensions. The axis index for the tensor is in [0, input.shape().dims()-1]. The function `flat_inner_outer_dims` expects an axis in [0, input.shape().dims()-1]. However, the code passes `axis_ - 1` which is in [-1, input.shape().dims()-2]. So when `axis_` is 0, we pass -1, which is invalid.
-      Therefore, the code is vulnerable.
-      However, note: the condition `axis_ &gt;= -1` and `axis_ &lt; input.shape().dims()` for non -1 does not prevent `axis_` from being 0. So the kernel will accept axis=0 and then crash.
-      Conclusion: YES, vulnerability detected.
-      But note: the problem says "vulnerable" meaning a security vulnerability. A crash is a vulnerability.
-      However, let's check if there is any other vulnerability.
-      Another point: the code uses `input_min_tensor.scalar&lt;T&gt;()` in the -1 branch. We have checked that the tensor is scalar (0 dimensions) so `scalar&lt;T&gt;()` is safe.
-      Also, the allocation of outputs: `ctx-&gt;allocate_output` uses the shape of the input (for `input_backprop`) and the shape of `input_min_tensor` (for the min and max backprops). Since we have validated the shapes (for the min and max tensors, we checked the dimensions and the size for the non -1 branch), the allocations are safe.
-      Therefore, the only vulnerability is the crash when `axis_` is 0.
-      So the answer is YES.
-      However, note: the problem might be that the condition for the axis in the non -1 branch should have been `axis_ &gt;= 0` (which it is) but the code should not subtract 1. The bug is in the code, not in the condition.
-      Therefore, we mark it as vulnerable.
-      But wait: the condition `axis_ &lt; input.shape().dims()` for non -1: the `input.shape().dims()` is the number of dimensions. The axis index for the tensor is 0-indexed, so the valid indices are 0 to `input.shape().dims()-1`. The code uses `axis_` as the axis index, but then subtracts 1. This is a mistake. The intended axis index for the tensor is `axis_`, so the code should not subtract 1.
-      So the vulnerability is due to a programming error that leads to an invalid axis index.
-      Therefore, the answer is YES.
-      However, note: the problem says "static program analysis". We are to decide based on the code. We found a bug that will cause a crash for a valid input (axis=0 for a 1D tensor). So it's a vulnerability.
-      Let's see if the condition `axis_ &lt; input.shape().dims()` is the same as the condition for the tensor axis? Yes, but the code uses `axis_ - 1` in the functor call, which is wrong.
-      So we are confident.
-      Answer: YES.
-      But note: the problem might be that the condition `axis_ &lt; input.shape().dims()` is not the same as the condition for the tensor axis? Actually, the condition is correct for the tensor axis (we require axis_ to be in [0, input.shape().dims()-1]), but the code then uses `axis_ - 1` which is not the axis we want.
-      Therefore, the vulnerability is present.
-      However, let's check the actual TensorFlow code for similar operations. In TensorFlow, the `QuantizeAndDequantize` op (or similar) might have a different implementation. But we are analyzing the provided code.
-      Given the provided code, we have to say YES.
-      But note: the problem says "vulnerable" meaning a security vulnerability. A crash is a vulnerability.
-      So we output YES.
-      However, let's consider: is it possible that the `flat_inner_outer_dims` function handles negative axis? The documentation of the function (if we had it) would tell. But in the absence of that, we assume that the function expects a non-negative axis. And the condition in the code (the `OP_REQUIRES` for the axis) does not prevent the negative axis in the function call.
-      Therefore, we mark it as vulnerable.
-      Final answer: YES.
-&lt;/think&gt;
-After a thorough static analysis of the provided code, the following vulnerability is identified:
+          <t>After a thorough static analysis of the provided code, the following vulnerability is identified:
 ### Vulnerability Analysis
 The code contains a **critical off-by-one error** in the `axis_ != -1` branch when `axis_` is 0. Specifically:
 1. The condition `OP_REQUIRES(ctx, (axis_ == -1 || axis_ &lt; input.shape().dims()), ...)` allows `axis_ = 0` (since `0 &lt; input.shape().dims()` is valid for tensors with ≥1 dimension).

</xml_diff>